<commit_message>
Updated code and docs, added shopping list file
</commit_message>
<xml_diff>
--- a/Electronic Components.xlsx
+++ b/Electronic Components.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cycho\source\repos\MyFYP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41D70D41-2053-4461-BDB4-14CA58CB777B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1145EC-8000-49BE-BF49-D9AE32C27D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9504" yWindow="1320" windowWidth="12672" windowHeight="9240" xr2:uid="{B27D4855-7488-4A18-9371-614F08F2D3ED}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Controller Components</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>13-20</t>
+  </si>
+  <si>
+    <t>330Ohm Resistors</t>
+  </si>
+  <si>
+    <t>Wire</t>
   </si>
 </sst>
 </file>
@@ -470,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{195C5795-F107-4B00-8355-277410C362DC}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" customWidth="1"/>
@@ -554,6 +560,19 @@
         <v>11</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>